<commit_message>
Added new RDF data schemes and visual schemes for economy-table116-120, fixed XLSX spreadsheets for economy-table117-120
</commit_message>
<xml_diff>
--- a/sources/table_normalization/xlsx/economy-table117.xlsx
+++ b/sources/table_normalization/xlsx/economy-table117.xlsx
@@ -383,7 +383,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="1">
-    <numFmt numFmtId="168" formatCode="#,##0,;\-#,##0,;\-"/>
+    <numFmt numFmtId="164" formatCode="#,##0,;\-#,##0,;\-"/>
   </numFmts>
   <fonts count="17">
     <font>
@@ -488,7 +488,7 @@
       <charset val="134"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -504,12 +504,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor indexed="24"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -600,7 +594,7 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0"/>
-    <xf numFmtId="168" fontId="16" fillId="0" borderId="0">
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0">
       <alignment wrapText="1"/>
       <protection locked="0"/>
     </xf>
@@ -611,7 +605,7 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyProtection="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
@@ -652,10 +646,6 @@
       <alignment horizontal="right" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="3" fontId="1" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
       <protection locked="0"/>
@@ -681,10 +671,6 @@
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="1" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="3" fontId="1" fillId="2" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
       <protection locked="0"/>
     </xf>
@@ -697,90 +683,110 @@
       <alignment horizontal="right" vertical="top" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="5" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="3" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="4" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="3" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="3" fontId="2" fillId="5" borderId="0" xfId="8" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="3" fontId="2" fillId="4" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <alignment wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="4" borderId="0" xfId="8" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="3" fontId="2" fillId="5" borderId="0" xfId="8" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="4" borderId="0" xfId="8" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="3" fontId="1" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="3" fontId="1" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="3" fontId="1" fillId="4" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="5" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="5" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="2" fillId="5" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="3" fontId="2" fillId="4" borderId="5" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="3" fontId="2" fillId="5" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
-      <alignment wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="3" fontId="4" fillId="4" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="3" fontId="4" fillId="4" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="3" fontId="1" fillId="6" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
       <protection locked="0"/>
     </xf>
   </cellXfs>
@@ -1927,28 +1933,28 @@
     </row>
     <row r="2" spans="1:224" s="1" customFormat="1">
       <c r="A2" s="6"/>
-      <c r="B2" s="36" t="s">
+      <c r="B2" s="27" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="36" t="s">
+      <c r="C2" s="27" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="36" t="s">
+      <c r="D2" s="27" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="36" t="s">
+      <c r="E2" s="27" t="s">
         <v>8</v>
       </c>
-      <c r="F2" s="36" t="s">
+      <c r="F2" s="27" t="s">
         <v>8</v>
       </c>
-      <c r="G2" s="36" t="s">
+      <c r="G2" s="27" t="s">
         <v>9</v>
       </c>
-      <c r="H2" s="36" t="s">
+      <c r="H2" s="27" t="s">
         <v>9</v>
       </c>
-      <c r="I2" s="36" t="s">
+      <c r="I2" s="27" t="s">
         <v>9</v>
       </c>
       <c r="J2" s="2"/>
@@ -2168,17 +2174,17 @@
       <c r="HP2" s="2"/>
     </row>
     <row r="3" spans="1:224" s="2" customFormat="1" ht="11.15" customHeight="1">
-      <c r="A3" s="48" t="s">
+      <c r="A3" s="42" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="49"/>
-      <c r="C3" s="49"/>
-      <c r="D3" s="49"/>
-      <c r="E3" s="49"/>
-      <c r="F3" s="49"/>
-      <c r="G3" s="49"/>
-      <c r="H3" s="49"/>
-      <c r="I3" s="49"/>
+      <c r="B3" s="45"/>
+      <c r="C3" s="45"/>
+      <c r="D3" s="45"/>
+      <c r="E3" s="45"/>
+      <c r="F3" s="45"/>
+      <c r="G3" s="45"/>
+      <c r="H3" s="45"/>
+      <c r="I3" s="45"/>
     </row>
     <row r="4" spans="1:224" s="3" customFormat="1" ht="11.15" customHeight="1">
       <c r="A4" s="9" t="s">
@@ -2897,31 +2903,31 @@
       <c r="HP6" s="5"/>
     </row>
     <row r="7" spans="1:224" s="4" customFormat="1" ht="11.15" customHeight="1">
-      <c r="A7" s="37" t="s">
+      <c r="A7" s="46" t="s">
         <v>14</v>
       </c>
-      <c r="B7" s="15">
+      <c r="B7" s="47">
         <v>300105</v>
       </c>
-      <c r="C7" s="15">
+      <c r="C7" s="47">
         <v>313275</v>
       </c>
-      <c r="D7" s="15">
+      <c r="D7" s="47">
         <v>333172</v>
       </c>
-      <c r="E7" s="15">
+      <c r="E7" s="47">
         <v>345844</v>
       </c>
-      <c r="F7" s="15">
+      <c r="F7" s="47">
         <v>340711</v>
       </c>
-      <c r="G7" s="15">
+      <c r="G7" s="47">
         <v>345300</v>
       </c>
-      <c r="H7" s="15">
+      <c r="H7" s="47">
         <v>348300</v>
       </c>
-      <c r="I7" s="15">
+      <c r="I7" s="47">
         <v>346300</v>
       </c>
     </row>
@@ -2935,22 +2941,22 @@
       <c r="C8" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="D8" s="16" t="s">
-        <v>16</v>
-      </c>
-      <c r="E8" s="16" t="s">
-        <v>16</v>
-      </c>
-      <c r="F8" s="16" t="s">
-        <v>16</v>
-      </c>
-      <c r="G8" s="16" t="s">
-        <v>16</v>
-      </c>
-      <c r="H8" s="16" t="s">
-        <v>16</v>
-      </c>
-      <c r="I8" s="16" t="s">
+      <c r="D8" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="E8" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="F8" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="G8" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="H8" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="I8" s="15" t="s">
         <v>16</v>
       </c>
     </row>
@@ -2964,27 +2970,27 @@
       <c r="C9" s="13">
         <v>150817</v>
       </c>
-      <c r="D9" s="17">
+      <c r="D9" s="16">
         <v>164048</v>
       </c>
-      <c r="E9" s="17">
+      <c r="E9" s="16">
         <v>169960</v>
       </c>
-      <c r="F9" s="17">
+      <c r="F9" s="16">
         <v>176029</v>
       </c>
-      <c r="G9" s="17">
+      <c r="G9" s="16">
         <v>183192</v>
       </c>
-      <c r="H9" s="17">
+      <c r="H9" s="16">
         <v>183259</v>
       </c>
-      <c r="I9" s="17">
+      <c r="I9" s="16">
         <v>186305</v>
       </c>
     </row>
     <row r="10" spans="1:224" ht="11.15" customHeight="1">
-      <c r="A10" s="18" t="s">
+      <c r="A10" s="17" t="s">
         <v>18</v>
       </c>
       <c r="B10" s="13">
@@ -2993,27 +2999,27 @@
       <c r="C10" s="13">
         <v>24154</v>
       </c>
-      <c r="D10" s="17">
+      <c r="D10" s="16">
         <v>27651</v>
       </c>
-      <c r="E10" s="17">
+      <c r="E10" s="16">
         <v>28924</v>
       </c>
-      <c r="F10" s="17">
+      <c r="F10" s="16">
         <v>29967</v>
       </c>
-      <c r="G10" s="17">
+      <c r="G10" s="16">
         <v>26141</v>
       </c>
-      <c r="H10" s="17">
+      <c r="H10" s="16">
         <v>26229</v>
       </c>
-      <c r="I10" s="17">
+      <c r="I10" s="16">
         <v>26656</v>
       </c>
     </row>
     <row r="11" spans="1:224" ht="11.15" customHeight="1">
-      <c r="A11" s="18" t="s">
+      <c r="A11" s="17" t="s">
         <v>19</v>
       </c>
       <c r="B11" s="13">
@@ -3022,22 +3028,22 @@
       <c r="C11" s="13">
         <v>5416</v>
       </c>
-      <c r="D11" s="17">
+      <c r="D11" s="16">
         <v>1532</v>
       </c>
-      <c r="E11" s="17">
+      <c r="E11" s="16">
         <v>-78069</v>
       </c>
-      <c r="F11" s="17">
+      <c r="F11" s="16">
         <v>6054</v>
       </c>
-      <c r="G11" s="17">
+      <c r="G11" s="16">
         <v>4998</v>
       </c>
-      <c r="H11" s="17">
+      <c r="H11" s="16">
         <v>865</v>
       </c>
-      <c r="I11" s="17">
+      <c r="I11" s="16">
         <v>1049</v>
       </c>
     </row>
@@ -3051,22 +3057,22 @@
       <c r="C12" s="13">
         <v>1011</v>
       </c>
-      <c r="D12" s="17">
+      <c r="D12" s="16">
         <v>1001</v>
       </c>
-      <c r="E12" s="17">
+      <c r="E12" s="16">
         <v>995</v>
       </c>
-      <c r="F12" s="17">
+      <c r="F12" s="16">
         <v>1399</v>
       </c>
-      <c r="G12" s="17">
+      <c r="G12" s="16">
         <v>1141</v>
       </c>
-      <c r="H12" s="17">
+      <c r="H12" s="16">
         <v>932</v>
       </c>
-      <c r="I12" s="17">
+      <c r="I12" s="16">
         <v>932</v>
       </c>
     </row>
@@ -3080,22 +3086,22 @@
       <c r="C13" s="13">
         <v>3316</v>
       </c>
-      <c r="D13" s="17">
+      <c r="D13" s="16">
         <v>3464</v>
       </c>
-      <c r="E13" s="17">
+      <c r="E13" s="16">
         <v>3303</v>
       </c>
-      <c r="F13" s="17">
+      <c r="F13" s="16">
         <v>3690</v>
       </c>
-      <c r="G13" s="17">
+      <c r="G13" s="16">
         <v>3868</v>
       </c>
-      <c r="H13" s="17">
+      <c r="H13" s="16">
         <v>3828</v>
       </c>
-      <c r="I13" s="17">
+      <c r="I13" s="16">
         <v>3826</v>
       </c>
     </row>
@@ -3109,22 +3115,22 @@
       <c r="C14" s="13">
         <v>-942</v>
       </c>
-      <c r="D14" s="17">
+      <c r="D14" s="16">
         <v>-233</v>
       </c>
-      <c r="E14" s="17">
+      <c r="E14" s="16">
         <v>-287</v>
       </c>
-      <c r="F14" s="17">
+      <c r="F14" s="16">
         <v>-624</v>
       </c>
-      <c r="G14" s="17">
+      <c r="G14" s="16">
         <v>-686</v>
       </c>
-      <c r="H14" s="17">
+      <c r="H14" s="16">
         <v>-1042</v>
       </c>
-      <c r="I14" s="17">
+      <c r="I14" s="16">
         <v>-1657</v>
       </c>
     </row>
@@ -3138,22 +3144,22 @@
       <c r="C15" s="13">
         <v>43085</v>
       </c>
-      <c r="D15" s="17">
+      <c r="D15" s="16">
         <v>44609</v>
       </c>
-      <c r="E15" s="17">
+      <c r="E15" s="16">
         <v>55509</v>
       </c>
-      <c r="F15" s="17">
+      <c r="F15" s="16">
         <v>50917</v>
       </c>
-      <c r="G15" s="17">
+      <c r="G15" s="16">
         <v>51021</v>
       </c>
-      <c r="H15" s="17">
+      <c r="H15" s="16">
         <v>41686</v>
       </c>
-      <c r="I15" s="17">
+      <c r="I15" s="16">
         <v>43428</v>
       </c>
     </row>
@@ -3167,13 +3173,13 @@
       <c r="C16" s="13">
         <v>41551</v>
       </c>
-      <c r="D16" s="17">
+      <c r="D16" s="16">
         <v>-27588</v>
       </c>
-      <c r="E16" s="17">
+      <c r="E16" s="16">
         <v>-14579</v>
       </c>
-      <c r="F16" s="17">
+      <c r="F16" s="16">
         <v>-16575</v>
       </c>
       <c r="G16" s="13" t="s">
@@ -3196,51 +3202,51 @@
       <c r="C17" s="13">
         <v>1765</v>
       </c>
-      <c r="D17" s="17">
+      <c r="D17" s="16">
         <v>2739</v>
       </c>
-      <c r="E17" s="17">
+      <c r="E17" s="16">
         <v>1111</v>
       </c>
-      <c r="F17" s="17">
+      <c r="F17" s="16">
         <v>200</v>
       </c>
-      <c r="G17" s="17">
+      <c r="G17" s="16">
         <v>4848</v>
       </c>
-      <c r="H17" s="17">
+      <c r="H17" s="16">
         <v>6176</v>
       </c>
-      <c r="I17" s="17">
+      <c r="I17" s="16">
         <v>6663</v>
       </c>
     </row>
     <row r="18" spans="1:9" s="4" customFormat="1" ht="11.15" customHeight="1">
-      <c r="A18" s="14" t="s">
+      <c r="A18" s="46" t="s">
         <v>27</v>
       </c>
-      <c r="B18" s="15">
+      <c r="B18" s="47">
         <v>218151</v>
       </c>
-      <c r="C18" s="15">
+      <c r="C18" s="47">
         <v>270173</v>
       </c>
-      <c r="D18" s="15">
+      <c r="D18" s="47">
         <v>217223</v>
       </c>
-      <c r="E18" s="15">
+      <c r="E18" s="47">
         <v>166869</v>
       </c>
-      <c r="F18" s="15">
+      <c r="F18" s="47">
         <v>251056</v>
       </c>
-      <c r="G18" s="15">
+      <c r="G18" s="47">
         <v>274523</v>
       </c>
-      <c r="H18" s="15">
+      <c r="H18" s="47">
         <v>261933</v>
       </c>
-      <c r="I18" s="15">
+      <c r="I18" s="47">
         <v>267202</v>
       </c>
     </row>
@@ -3248,33 +3254,33 @@
       <c r="A19" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="B19" s="19" t="s">
-        <v>16</v>
-      </c>
-      <c r="C19" s="19" t="s">
-        <v>16</v>
-      </c>
-      <c r="D19" s="20" t="s">
-        <v>16</v>
-      </c>
-      <c r="E19" s="20" t="s">
-        <v>16</v>
-      </c>
-      <c r="F19" s="20" t="s">
-        <v>16</v>
-      </c>
-      <c r="G19" s="20" t="s">
-        <v>16</v>
-      </c>
-      <c r="H19" s="20" t="s">
-        <v>16</v>
-      </c>
-      <c r="I19" s="20" t="s">
+      <c r="B19" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="C19" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="D19" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="E19" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="F19" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="G19" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="H19" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="I19" s="19" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="20" spans="1:9" ht="11.15" customHeight="1">
-      <c r="A20" s="21" t="s">
+      <c r="A20" s="20" t="s">
         <v>29</v>
       </c>
       <c r="B20" s="13">
@@ -3283,27 +3289,27 @@
       <c r="C20" s="13">
         <v>3060</v>
       </c>
-      <c r="D20" s="17">
+      <c r="D20" s="16">
         <v>6419</v>
       </c>
-      <c r="E20" s="17">
+      <c r="E20" s="16">
         <v>8414</v>
       </c>
-      <c r="F20" s="17">
+      <c r="F20" s="16">
         <v>7702</v>
       </c>
-      <c r="G20" s="17">
+      <c r="G20" s="16">
         <v>7477</v>
       </c>
-      <c r="H20" s="17">
+      <c r="H20" s="16">
         <v>8670</v>
       </c>
-      <c r="I20" s="17">
+      <c r="I20" s="16">
         <v>9562</v>
       </c>
     </row>
     <row r="21" spans="1:9" ht="11.15" customHeight="1">
-      <c r="A21" s="21" t="s">
+      <c r="A21" s="20" t="s">
         <v>30</v>
       </c>
       <c r="B21" s="13">
@@ -3312,22 +3318,22 @@
       <c r="C21" s="13">
         <v>26966</v>
       </c>
-      <c r="D21" s="17">
+      <c r="D21" s="16">
         <v>25794</v>
       </c>
-      <c r="E21" s="17">
+      <c r="E21" s="16">
         <v>22906</v>
       </c>
-      <c r="F21" s="17">
+      <c r="F21" s="16">
         <v>26740</v>
       </c>
-      <c r="G21" s="17">
+      <c r="G21" s="16">
         <v>27330</v>
       </c>
-      <c r="H21" s="17">
+      <c r="H21" s="16">
         <v>28742</v>
       </c>
-      <c r="I21" s="17">
+      <c r="I21" s="16">
         <v>30051</v>
       </c>
     </row>
@@ -3341,22 +3347,22 @@
       <c r="C22" s="13">
         <v>30300</v>
       </c>
-      <c r="D22" s="17">
+      <c r="D22" s="16">
         <v>30185</v>
       </c>
-      <c r="E22" s="17">
+      <c r="E22" s="16">
         <v>44399</v>
       </c>
-      <c r="F22" s="17">
+      <c r="F22" s="16">
         <v>46976</v>
       </c>
-      <c r="G22" s="17">
+      <c r="G22" s="16">
         <v>44788</v>
       </c>
-      <c r="H22" s="17">
+      <c r="H22" s="16">
         <v>46123</v>
       </c>
-      <c r="I22" s="17">
+      <c r="I22" s="16">
         <v>53224</v>
       </c>
     </row>
@@ -3370,143 +3376,143 @@
       <c r="C23" s="13">
         <v>-79045</v>
       </c>
-      <c r="D23" s="17">
+      <c r="D23" s="16">
         <v>-10489</v>
       </c>
-      <c r="E23" s="17">
+      <c r="E23" s="16">
         <v>42932</v>
       </c>
-      <c r="F23" s="17">
+      <c r="F23" s="16">
         <v>-27497</v>
       </c>
-      <c r="G23" s="17">
+      <c r="G23" s="16">
         <f>-35400+640</f>
         <v>-34760</v>
       </c>
-      <c r="H23" s="17">
+      <c r="H23" s="16">
         <f>-19305-1000</f>
         <v>-20305</v>
       </c>
-      <c r="I23" s="17">
+      <c r="I23" s="16">
         <f>-20005</f>
         <v>-20005</v>
       </c>
     </row>
     <row r="24" spans="1:9" s="4" customFormat="1" ht="13" customHeight="1">
-      <c r="A24" s="38" t="s">
+      <c r="A24" s="48" t="s">
         <v>33</v>
       </c>
-      <c r="B24" s="22">
+      <c r="B24" s="49">
         <v>17910</v>
       </c>
-      <c r="C24" s="22">
+      <c r="C24" s="49">
         <v>-18719</v>
       </c>
-      <c r="D24" s="22">
+      <c r="D24" s="49">
         <v>51909</v>
       </c>
-      <c r="E24" s="22">
+      <c r="E24" s="49">
         <v>118651</v>
       </c>
-      <c r="F24" s="22">
+      <c r="F24" s="49">
         <v>53921</v>
       </c>
-      <c r="G24" s="22">
+      <c r="G24" s="49">
         <f>44194+640</f>
         <v>44834</v>
       </c>
-      <c r="H24" s="22">
+      <c r="H24" s="49">
         <f>64229-1000</f>
         <v>63229</v>
       </c>
-      <c r="I24" s="22">
+      <c r="I24" s="49">
         <f>72831</f>
         <v>72831</v>
       </c>
     </row>
     <row r="25" spans="1:9" s="4" customFormat="1" ht="13" customHeight="1">
-      <c r="A25" s="39" t="s">
+      <c r="A25" s="50" t="s">
         <v>34</v>
       </c>
-      <c r="B25" s="23">
+      <c r="B25" s="51">
         <v>236060</v>
       </c>
-      <c r="C25" s="23">
+      <c r="C25" s="51">
         <v>251453</v>
       </c>
-      <c r="D25" s="23">
+      <c r="D25" s="51">
         <v>269132</v>
       </c>
-      <c r="E25" s="23">
+      <c r="E25" s="51">
         <v>285520</v>
       </c>
-      <c r="F25" s="23">
+      <c r="F25" s="51">
         <v>304977</v>
       </c>
-      <c r="G25" s="23">
+      <c r="G25" s="51">
         <f>318717+640</f>
         <v>319357</v>
       </c>
-      <c r="H25" s="23">
+      <c r="H25" s="51">
         <f>326162-1000</f>
         <v>325162</v>
       </c>
-      <c r="I25" s="23">
+      <c r="I25" s="51">
         <f>340033</f>
         <v>340033</v>
       </c>
     </row>
     <row r="26" spans="1:9" s="4" customFormat="1" ht="13" customHeight="1">
-      <c r="A26" s="40" t="s">
+      <c r="A26" s="30" t="s">
         <v>35</v>
       </c>
-      <c r="B26" s="24">
+      <c r="B26" s="22">
         <v>536165</v>
       </c>
-      <c r="C26" s="24">
+      <c r="C26" s="22">
         <v>564728</v>
       </c>
-      <c r="D26" s="24">
+      <c r="D26" s="22">
         <v>602304</v>
       </c>
-      <c r="E26" s="24">
+      <c r="E26" s="22">
         <v>631364</v>
       </c>
-      <c r="F26" s="24">
+      <c r="F26" s="22">
         <v>645688</v>
       </c>
-      <c r="G26" s="24">
+      <c r="G26" s="22">
         <v>664600</v>
       </c>
-      <c r="H26" s="24">
+      <c r="H26" s="22">
         <v>673600</v>
       </c>
-      <c r="I26" s="24">
+      <c r="I26" s="22">
         <v>686400</v>
       </c>
     </row>
     <row r="27" spans="1:9" s="2" customFormat="1" ht="11.15" customHeight="1">
-      <c r="A27" s="48" t="s">
+      <c r="A27" s="42" t="s">
         <v>36</v>
       </c>
-      <c r="B27" s="50" t="s">
-        <v>16</v>
-      </c>
-      <c r="C27" s="50" t="s">
-        <v>16</v>
-      </c>
-      <c r="D27" s="51" t="s">
-        <v>16</v>
-      </c>
-      <c r="E27" s="51" t="s">
-        <v>16</v>
-      </c>
-      <c r="F27" s="51" t="s">
-        <v>16</v>
-      </c>
-      <c r="G27" s="51"/>
-      <c r="H27" s="51"/>
-      <c r="I27" s="51"/>
+      <c r="B27" s="43" t="s">
+        <v>16</v>
+      </c>
+      <c r="C27" s="43" t="s">
+        <v>16</v>
+      </c>
+      <c r="D27" s="44" t="s">
+        <v>16</v>
+      </c>
+      <c r="E27" s="44" t="s">
+        <v>16</v>
+      </c>
+      <c r="F27" s="44" t="s">
+        <v>16</v>
+      </c>
+      <c r="G27" s="44"/>
+      <c r="H27" s="44"/>
+      <c r="I27" s="44"/>
     </row>
     <row r="28" spans="1:9" ht="11.15" customHeight="1">
       <c r="A28" s="9" t="s">
@@ -3518,45 +3524,45 @@
       <c r="C28" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="D28" s="16" t="s">
-        <v>16</v>
-      </c>
-      <c r="E28" s="16" t="s">
-        <v>16</v>
-      </c>
-      <c r="F28" s="16" t="s">
-        <v>16</v>
-      </c>
-      <c r="G28" s="16"/>
-      <c r="H28" s="16"/>
-      <c r="I28" s="16"/>
+      <c r="D28" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="E28" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="F28" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="G28" s="15"/>
+      <c r="H28" s="15"/>
+      <c r="I28" s="15"/>
     </row>
     <row r="29" spans="1:9" s="4" customFormat="1" ht="13" customHeight="1">
       <c r="A29" s="52" t="s">
         <v>38</v>
       </c>
-      <c r="B29" s="15">
+      <c r="B29" s="47">
         <v>44821</v>
       </c>
-      <c r="C29" s="15">
+      <c r="C29" s="47">
         <v>48511</v>
       </c>
-      <c r="D29" s="15">
+      <c r="D29" s="47">
         <v>56959</v>
       </c>
-      <c r="E29" s="15">
+      <c r="E29" s="47">
         <v>49815</v>
       </c>
-      <c r="F29" s="15">
+      <c r="F29" s="47">
         <v>42156</v>
       </c>
-      <c r="G29" s="15">
+      <c r="G29" s="47">
         <v>43800</v>
       </c>
-      <c r="H29" s="15">
+      <c r="H29" s="47">
         <v>40900</v>
       </c>
-      <c r="I29" s="15">
+      <c r="I29" s="47">
         <v>41300</v>
       </c>
     </row>
@@ -3570,22 +3576,22 @@
       <c r="C30" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="D30" s="17" t="s">
-        <v>16</v>
-      </c>
-      <c r="E30" s="17" t="s">
-        <v>16</v>
-      </c>
-      <c r="F30" s="17" t="s">
-        <v>16</v>
-      </c>
-      <c r="G30" s="17" t="s">
-        <v>16</v>
-      </c>
-      <c r="H30" s="17" t="s">
-        <v>16</v>
-      </c>
-      <c r="I30" s="17" t="s">
+      <c r="D30" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="E30" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="F30" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="G30" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="H30" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="I30" s="16" t="s">
         <v>16</v>
       </c>
     </row>
@@ -3599,22 +3605,22 @@
       <c r="C31" s="13">
         <v>536</v>
       </c>
-      <c r="D31" s="17">
+      <c r="D31" s="16">
         <v>752</v>
       </c>
-      <c r="E31" s="17">
+      <c r="E31" s="16">
         <v>597</v>
       </c>
-      <c r="F31" s="17">
+      <c r="F31" s="16">
         <v>404</v>
       </c>
-      <c r="G31" s="17">
+      <c r="G31" s="16">
         <v>712</v>
       </c>
-      <c r="H31" s="17">
+      <c r="H31" s="16">
         <v>497</v>
       </c>
-      <c r="I31" s="17">
+      <c r="I31" s="16">
         <v>568</v>
       </c>
     </row>
@@ -3628,22 +3634,22 @@
       <c r="C32" s="13">
         <v>81</v>
       </c>
-      <c r="D32" s="17">
+      <c r="D32" s="16">
         <v>123</v>
       </c>
-      <c r="E32" s="17">
+      <c r="E32" s="16">
         <v>114</v>
       </c>
-      <c r="F32" s="17">
+      <c r="F32" s="16">
         <v>191</v>
       </c>
-      <c r="G32" s="17">
+      <c r="G32" s="16">
         <v>54</v>
       </c>
-      <c r="H32" s="17">
+      <c r="H32" s="16">
         <v>177</v>
       </c>
-      <c r="I32" s="17">
+      <c r="I32" s="16">
         <v>145</v>
       </c>
     </row>
@@ -3657,22 +3663,22 @@
       <c r="C33" s="13">
         <v>4330</v>
       </c>
-      <c r="D33" s="17">
+      <c r="D33" s="16">
         <v>4408</v>
       </c>
-      <c r="E33" s="17">
+      <c r="E33" s="16">
         <v>4778</v>
       </c>
-      <c r="F33" s="17">
+      <c r="F33" s="16">
         <v>5646</v>
       </c>
-      <c r="G33" s="17">
+      <c r="G33" s="16">
         <v>6603</v>
       </c>
-      <c r="H33" s="17">
+      <c r="H33" s="16">
         <v>8592</v>
       </c>
-      <c r="I33" s="17">
+      <c r="I33" s="16">
         <v>10440</v>
       </c>
     </row>
@@ -3686,13 +3692,13 @@
       <c r="C34" s="13">
         <v>85525</v>
       </c>
-      <c r="D34" s="17">
+      <c r="D34" s="16">
         <v>38330</v>
       </c>
-      <c r="E34" s="17">
+      <c r="E34" s="16">
         <v>-2984</v>
       </c>
-      <c r="F34" s="17">
+      <c r="F34" s="16">
         <v>-3721</v>
       </c>
       <c r="G34" s="13" t="s">
@@ -3706,7 +3712,7 @@
       </c>
     </row>
     <row r="35" spans="1:9" ht="11.15" customHeight="1">
-      <c r="A35" s="25" t="s">
+      <c r="A35" s="23" t="s">
         <v>26</v>
       </c>
       <c r="B35" s="13">
@@ -3715,51 +3721,51 @@
       <c r="C35" s="13">
         <v>393</v>
       </c>
-      <c r="D35" s="17">
+      <c r="D35" s="16">
         <v>4082</v>
       </c>
-      <c r="E35" s="17">
+      <c r="E35" s="16">
         <v>1297</v>
       </c>
-      <c r="F35" s="17">
+      <c r="F35" s="16">
         <v>967</v>
       </c>
-      <c r="G35" s="17">
+      <c r="G35" s="16">
         <v>2829</v>
       </c>
-      <c r="H35" s="17">
+      <c r="H35" s="16">
         <v>2834</v>
       </c>
-      <c r="I35" s="17">
+      <c r="I35" s="16">
         <v>2735</v>
       </c>
     </row>
     <row r="36" spans="1:9" s="4" customFormat="1" ht="13" customHeight="1">
-      <c r="A36" s="37" t="s">
+      <c r="A36" s="46" t="s">
         <v>40</v>
       </c>
-      <c r="B36" s="15">
+      <c r="B36" s="47">
         <v>6005</v>
       </c>
-      <c r="C36" s="15">
+      <c r="C36" s="47">
         <v>90866</v>
       </c>
-      <c r="D36" s="15">
+      <c r="D36" s="47">
         <v>47694</v>
       </c>
-      <c r="E36" s="15">
+      <c r="E36" s="47">
         <v>3802</v>
       </c>
-      <c r="F36" s="15">
+      <c r="F36" s="47">
         <v>3488</v>
       </c>
-      <c r="G36" s="15">
+      <c r="G36" s="47">
         <v>10198</v>
       </c>
-      <c r="H36" s="15">
+      <c r="H36" s="47">
         <v>12100</v>
       </c>
-      <c r="I36" s="15">
+      <c r="I36" s="47">
         <v>13888</v>
       </c>
     </row>
@@ -3773,22 +3779,22 @@
       <c r="C37" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="D37" s="17" t="s">
-        <v>16</v>
-      </c>
-      <c r="E37" s="17" t="s">
-        <v>16</v>
-      </c>
-      <c r="F37" s="17" t="s">
-        <v>16</v>
-      </c>
-      <c r="G37" s="17" t="s">
-        <v>16</v>
-      </c>
-      <c r="H37" s="17" t="s">
+      <c r="D37" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="E37" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="F37" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="G37" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="H37" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="I37" s="17" t="s">
+      <c r="I37" s="16" t="s">
         <v>16</v>
       </c>
     </row>
@@ -3802,27 +3808,27 @@
       <c r="C38" s="13">
         <v>7321</v>
       </c>
-      <c r="D38" s="17">
+      <c r="D38" s="16">
         <v>5241</v>
       </c>
-      <c r="E38" s="17">
+      <c r="E38" s="16">
         <v>5448</v>
       </c>
-      <c r="F38" s="17">
+      <c r="F38" s="16">
         <v>13641</v>
       </c>
-      <c r="G38" s="17">
+      <c r="G38" s="16">
         <v>5268</v>
       </c>
-      <c r="H38" s="17">
+      <c r="H38" s="16">
         <v>4921</v>
       </c>
-      <c r="I38" s="17">
+      <c r="I38" s="16">
         <v>4815</v>
       </c>
     </row>
     <row r="39" spans="1:9" ht="11.15" customHeight="1">
-      <c r="A39" s="21" t="s">
+      <c r="A39" s="20" t="s">
         <v>43</v>
       </c>
       <c r="B39" s="13">
@@ -3831,22 +3837,22 @@
       <c r="C39" s="13">
         <v>7294</v>
       </c>
-      <c r="D39" s="17">
+      <c r="D39" s="16">
         <v>7983</v>
       </c>
-      <c r="E39" s="17">
+      <c r="E39" s="16">
         <v>8137</v>
       </c>
-      <c r="F39" s="17">
+      <c r="F39" s="16">
         <v>6115</v>
       </c>
-      <c r="G39" s="17">
+      <c r="G39" s="16">
         <v>6244</v>
       </c>
-      <c r="H39" s="17">
+      <c r="H39" s="16">
         <v>5734</v>
       </c>
-      <c r="I39" s="17">
+      <c r="I39" s="16">
         <v>5339</v>
       </c>
     </row>
@@ -3860,117 +3866,117 @@
       <c r="C40" s="13">
         <v>-88975</v>
       </c>
-      <c r="D40" s="17">
+      <c r="D40" s="16">
         <v>-50032</v>
       </c>
-      <c r="E40" s="17">
+      <c r="E40" s="16">
         <v>-8932</v>
       </c>
-      <c r="F40" s="17">
+      <c r="F40" s="16">
         <v>-16201</v>
       </c>
-      <c r="G40" s="17">
+      <c r="G40" s="16">
         <f>-47008+228</f>
         <v>-46780</v>
       </c>
-      <c r="H40" s="17">
+      <c r="H40" s="16">
         <v>-17187</v>
       </c>
-      <c r="I40" s="17">
+      <c r="I40" s="16">
         <v>-18411</v>
       </c>
     </row>
     <row r="41" spans="1:9" s="4" customFormat="1" ht="11.25" customHeight="1">
-      <c r="A41" s="38" t="s">
+      <c r="A41" s="48" t="s">
         <v>44</v>
       </c>
-      <c r="B41" s="22">
+      <c r="B41" s="49">
         <v>-4055</v>
       </c>
-      <c r="C41" s="22">
+      <c r="C41" s="49">
         <v>-74359</v>
       </c>
-      <c r="D41" s="22">
+      <c r="D41" s="49">
         <v>-36808</v>
       </c>
-      <c r="E41" s="22">
+      <c r="E41" s="49">
         <v>4653</v>
       </c>
-      <c r="F41" s="22">
+      <c r="F41" s="49">
         <v>3556</v>
       </c>
-      <c r="G41" s="22">
+      <c r="G41" s="49">
         <f>-35497+228</f>
         <v>-35269</v>
       </c>
-      <c r="H41" s="22">
+      <c r="H41" s="49">
         <v>-6532</v>
       </c>
-      <c r="I41" s="22">
+      <c r="I41" s="49">
         <v>-8256</v>
       </c>
     </row>
     <row r="42" spans="1:9" s="4" customFormat="1" ht="11.25" customHeight="1">
-      <c r="A42" s="38" t="s">
+      <c r="A42" s="48" t="s">
         <v>45</v>
       </c>
-      <c r="B42" s="22">
+      <c r="B42" s="49">
         <v>1951</v>
       </c>
-      <c r="C42" s="22">
+      <c r="C42" s="49">
         <v>16506</v>
       </c>
-      <c r="D42" s="22">
+      <c r="D42" s="49">
         <v>10887</v>
       </c>
-      <c r="E42" s="22">
+      <c r="E42" s="49">
         <v>8455</v>
       </c>
-      <c r="F42" s="22">
+      <c r="F42" s="49">
         <v>7044</v>
       </c>
-      <c r="G42" s="22">
+      <c r="G42" s="49">
         <f>-25299+228</f>
         <v>-25071</v>
       </c>
-      <c r="H42" s="22">
+      <c r="H42" s="49">
         <v>5568</v>
       </c>
-      <c r="I42" s="22">
+      <c r="I42" s="49">
         <v>5632</v>
       </c>
     </row>
     <row r="43" spans="1:9" s="4" customFormat="1" ht="11.25" customHeight="1">
-      <c r="A43" s="37" t="s">
+      <c r="A43" s="28" t="s">
         <v>57</v>
       </c>
-      <c r="B43" s="15">
+      <c r="B43" s="14">
         <v>46772</v>
       </c>
-      <c r="C43" s="15">
+      <c r="C43" s="14">
         <v>65017</v>
       </c>
-      <c r="D43" s="15">
+      <c r="D43" s="14">
         <v>67846</v>
       </c>
-      <c r="E43" s="15">
+      <c r="E43" s="14">
         <v>58270</v>
       </c>
-      <c r="F43" s="15">
+      <c r="F43" s="14">
         <v>49200</v>
       </c>
-      <c r="G43" s="15">
+      <c r="G43" s="14">
         <v>18600</v>
       </c>
-      <c r="H43" s="15">
+      <c r="H43" s="14">
         <v>46400</v>
       </c>
-      <c r="I43" s="15">
+      <c r="I43" s="14">
         <v>47000</v>
       </c>
     </row>
     <row r="44" spans="1:9" ht="11.25" customHeight="1">
-      <c r="A44" s="41" t="s">
+      <c r="A44" s="31" t="s">
         <v>56</v>
       </c>
       <c r="B44" s="13">
@@ -3979,276 +3985,276 @@
       <c r="C44" s="13">
         <v>18636</v>
       </c>
-      <c r="D44" s="17">
+      <c r="D44" s="16">
         <v>19335</v>
       </c>
-      <c r="E44" s="17">
+      <c r="E44" s="16">
         <v>20300</v>
       </c>
-      <c r="F44" s="17">
+      <c r="F44" s="16">
         <v>21121</v>
       </c>
-      <c r="G44" s="17">
+      <c r="G44" s="16">
         <v>22200</v>
       </c>
-      <c r="H44" s="17">
+      <c r="H44" s="16">
         <v>23056</v>
       </c>
-      <c r="I44" s="17">
+      <c r="I44" s="16">
         <v>23896</v>
       </c>
     </row>
     <row r="45" spans="1:9" s="4" customFormat="1" ht="11.25" customHeight="1">
-      <c r="A45" s="38" t="s">
+      <c r="A45" s="29" t="s">
         <v>58</v>
       </c>
-      <c r="B45" s="22">
+      <c r="B45" s="21">
         <v>29103</v>
       </c>
-      <c r="C45" s="22">
+      <c r="C45" s="21">
         <v>46381</v>
       </c>
-      <c r="D45" s="22">
+      <c r="D45" s="21">
         <v>48511</v>
       </c>
-      <c r="E45" s="22">
+      <c r="E45" s="21">
         <v>37970</v>
       </c>
-      <c r="F45" s="22">
+      <c r="F45" s="21">
         <v>28079</v>
       </c>
-      <c r="G45" s="22">
+      <c r="G45" s="21">
         <v>-3600</v>
       </c>
-      <c r="H45" s="22">
+      <c r="H45" s="21">
         <v>23400</v>
       </c>
-      <c r="I45" s="22">
+      <c r="I45" s="21">
         <v>23100</v>
       </c>
     </row>
     <row r="46" spans="1:9" s="4" customFormat="1" ht="13" customHeight="1">
-      <c r="A46" s="42" t="s">
+      <c r="A46" s="32" t="s">
         <v>59</v>
       </c>
-      <c r="B46" s="26">
+      <c r="B46" s="24">
         <v>582937</v>
       </c>
-      <c r="C46" s="26">
+      <c r="C46" s="24">
         <v>629745</v>
       </c>
-      <c r="D46" s="26">
+      <c r="D46" s="24">
         <v>670150</v>
       </c>
-      <c r="E46" s="26">
+      <c r="E46" s="24">
         <v>689634</v>
       </c>
-      <c r="F46" s="26">
+      <c r="F46" s="24">
         <v>694888</v>
       </c>
-      <c r="G46" s="26">
+      <c r="G46" s="24">
         <v>683400</v>
       </c>
-      <c r="H46" s="26">
+      <c r="H46" s="24">
         <v>720000</v>
       </c>
-      <c r="I46" s="26">
+      <c r="I46" s="24">
         <v>733500</v>
       </c>
     </row>
     <row r="47" spans="1:9" ht="11.15" customHeight="1">
-      <c r="A47" s="43" t="s">
+      <c r="A47" s="33" t="s">
         <v>46</v>
       </c>
-      <c r="B47" s="46" t="s">
-        <v>16</v>
-      </c>
-      <c r="C47" s="46" t="s">
-        <v>16</v>
-      </c>
-      <c r="D47" s="47" t="s">
-        <v>16</v>
-      </c>
-      <c r="E47" s="47" t="s">
-        <v>16</v>
-      </c>
-      <c r="F47" s="47" t="s">
-        <v>16</v>
-      </c>
-      <c r="G47" s="47" t="s">
-        <v>16</v>
-      </c>
-      <c r="H47" s="47" t="s">
-        <v>16</v>
-      </c>
-      <c r="I47" s="47" t="s">
+      <c r="B47" s="34" t="s">
+        <v>16</v>
+      </c>
+      <c r="C47" s="34" t="s">
+        <v>16</v>
+      </c>
+      <c r="D47" s="35" t="s">
+        <v>16</v>
+      </c>
+      <c r="E47" s="35" t="s">
+        <v>16</v>
+      </c>
+      <c r="F47" s="35" t="s">
+        <v>16</v>
+      </c>
+      <c r="G47" s="35" t="s">
+        <v>16</v>
+      </c>
+      <c r="H47" s="35" t="s">
+        <v>16</v>
+      </c>
+      <c r="I47" s="35" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="48" spans="1:9" ht="11.15" customHeight="1">
-      <c r="A48" s="44" t="s">
+      <c r="A48" s="53" t="s">
         <v>47</v>
       </c>
-      <c r="B48" s="13">
+      <c r="B48" s="34">
         <v>333142</v>
       </c>
-      <c r="C48" s="13">
+      <c r="C48" s="34">
         <v>349396</v>
       </c>
-      <c r="D48" s="13">
+      <c r="D48" s="34">
         <v>376288</v>
       </c>
-      <c r="E48" s="13">
+      <c r="E48" s="34">
         <v>375061</v>
       </c>
-      <c r="F48" s="13">
+      <c r="F48" s="34">
         <v>364015</v>
       </c>
-      <c r="G48" s="13">
+      <c r="G48" s="34">
         <v>371000</v>
       </c>
-      <c r="H48" s="13">
+      <c r="H48" s="34">
         <v>371100</v>
       </c>
-      <c r="I48" s="13">
+      <c r="I48" s="34">
         <v>368300</v>
       </c>
     </row>
     <row r="49" spans="1:9" ht="11.15" customHeight="1">
-      <c r="A49" s="44" t="s">
+      <c r="A49" s="53" t="s">
         <v>48</v>
       </c>
-      <c r="B49" s="13">
+      <c r="B49" s="34">
         <v>224156</v>
       </c>
-      <c r="C49" s="13">
+      <c r="C49" s="34">
         <v>361039</v>
       </c>
-      <c r="D49" s="17">
+      <c r="D49" s="35">
         <v>264918</v>
       </c>
-      <c r="E49" s="17">
+      <c r="E49" s="35">
         <v>170671</v>
       </c>
-      <c r="F49" s="17">
+      <c r="F49" s="35">
         <v>254544</v>
       </c>
-      <c r="G49" s="17">
+      <c r="G49" s="35">
         <v>284721</v>
       </c>
-      <c r="H49" s="17">
+      <c r="H49" s="35">
         <v>274032</v>
       </c>
-      <c r="I49" s="17">
+      <c r="I49" s="35">
         <v>281090</v>
       </c>
     </row>
     <row r="50" spans="1:9" ht="11.15" customHeight="1">
-      <c r="A50" s="45" t="s">
+      <c r="A50" s="54" t="s">
         <v>49</v>
       </c>
-      <c r="B50" s="27">
+      <c r="B50" s="55">
         <v>25639</v>
       </c>
-      <c r="C50" s="27">
+      <c r="C50" s="55">
         <v>-80690</v>
       </c>
-      <c r="D50" s="27">
+      <c r="D50" s="55">
         <v>28944</v>
       </c>
-      <c r="E50" s="27">
+      <c r="E50" s="55">
         <v>143902</v>
       </c>
-      <c r="F50" s="27">
+      <c r="F50" s="55">
         <v>76329</v>
       </c>
-      <c r="G50" s="27">
+      <c r="G50" s="55">
         <v>27665</v>
       </c>
-      <c r="H50" s="27">
+      <c r="H50" s="55">
         <v>74797</v>
       </c>
-      <c r="I50" s="27">
+      <c r="I50" s="55">
         <v>83775</v>
       </c>
     </row>
     <row r="51" spans="1:9" ht="11.25" customHeight="1">
-      <c r="A51" s="30" t="s">
+      <c r="A51" s="37" t="s">
         <v>50</v>
       </c>
-      <c r="B51" s="31"/>
-      <c r="C51" s="31"/>
-      <c r="D51" s="31"/>
-      <c r="E51" s="31"/>
-      <c r="F51" s="31"/>
-      <c r="G51" s="31"/>
-      <c r="H51" s="31"/>
-      <c r="I51" s="31"/>
+      <c r="B51" s="38"/>
+      <c r="C51" s="38"/>
+      <c r="D51" s="38"/>
+      <c r="E51" s="38"/>
+      <c r="F51" s="38"/>
+      <c r="G51" s="38"/>
+      <c r="H51" s="38"/>
+      <c r="I51" s="38"/>
     </row>
     <row r="52" spans="1:9" ht="11.25" customHeight="1">
-      <c r="A52" s="32" t="s">
+      <c r="A52" s="39" t="s">
         <v>51</v>
       </c>
-      <c r="B52" s="32"/>
-      <c r="C52" s="32"/>
-      <c r="D52" s="32"/>
-      <c r="E52" s="32"/>
-      <c r="F52" s="32"/>
-      <c r="G52" s="32"/>
-      <c r="H52" s="32"/>
-      <c r="I52" s="32"/>
+      <c r="B52" s="39"/>
+      <c r="C52" s="39"/>
+      <c r="D52" s="39"/>
+      <c r="E52" s="39"/>
+      <c r="F52" s="39"/>
+      <c r="G52" s="39"/>
+      <c r="H52" s="39"/>
+      <c r="I52" s="39"/>
     </row>
     <row r="53" spans="1:9" ht="11.25" customHeight="1">
-      <c r="A53" s="33" t="s">
+      <c r="A53" s="36" t="s">
         <v>52</v>
       </c>
-      <c r="B53" s="33"/>
-      <c r="C53" s="33"/>
-      <c r="D53" s="33"/>
-      <c r="E53" s="33"/>
-      <c r="F53" s="33"/>
-      <c r="G53" s="33"/>
-      <c r="H53" s="33"/>
-      <c r="I53" s="33"/>
+      <c r="B53" s="36"/>
+      <c r="C53" s="36"/>
+      <c r="D53" s="36"/>
+      <c r="E53" s="36"/>
+      <c r="F53" s="36"/>
+      <c r="G53" s="36"/>
+      <c r="H53" s="36"/>
+      <c r="I53" s="36"/>
     </row>
     <row r="54" spans="1:9" ht="11.25" customHeight="1">
-      <c r="A54" s="34" t="s">
+      <c r="A54" s="40" t="s">
         <v>53</v>
       </c>
-      <c r="B54" s="35"/>
-      <c r="C54" s="35"/>
-      <c r="D54" s="35"/>
-      <c r="E54" s="35"/>
-      <c r="F54" s="35"/>
-      <c r="G54" s="35"/>
-      <c r="H54" s="35"/>
-      <c r="I54" s="35"/>
+      <c r="B54" s="41"/>
+      <c r="C54" s="41"/>
+      <c r="D54" s="41"/>
+      <c r="E54" s="41"/>
+      <c r="F54" s="41"/>
+      <c r="G54" s="41"/>
+      <c r="H54" s="41"/>
+      <c r="I54" s="41"/>
     </row>
     <row r="55" spans="1:9" ht="11.25" customHeight="1">
-      <c r="A55" s="34" t="s">
+      <c r="A55" s="40" t="s">
         <v>54</v>
       </c>
-      <c r="B55" s="35"/>
-      <c r="C55" s="35"/>
-      <c r="D55" s="35"/>
-      <c r="E55" s="35"/>
-      <c r="F55" s="35"/>
-      <c r="G55" s="35"/>
-      <c r="H55" s="35"/>
-      <c r="I55" s="35"/>
+      <c r="B55" s="41"/>
+      <c r="C55" s="41"/>
+      <c r="D55" s="41"/>
+      <c r="E55" s="41"/>
+      <c r="F55" s="41"/>
+      <c r="G55" s="41"/>
+      <c r="H55" s="41"/>
+      <c r="I55" s="41"/>
     </row>
     <row r="56" spans="1:9" ht="11.25" customHeight="1">
-      <c r="A56" s="33" t="s">
+      <c r="A56" s="36" t="s">
         <v>55</v>
       </c>
-      <c r="B56" s="33"/>
-      <c r="C56" s="33"/>
-      <c r="D56" s="33"/>
-      <c r="E56" s="33"/>
-      <c r="F56" s="33"/>
-      <c r="G56" s="33"/>
-      <c r="H56" s="33"/>
-      <c r="I56" s="33"/>
+      <c r="B56" s="36"/>
+      <c r="C56" s="36"/>
+      <c r="D56" s="36"/>
+      <c r="E56" s="36"/>
+      <c r="F56" s="36"/>
+      <c r="G56" s="36"/>
+      <c r="H56" s="36"/>
+      <c r="I56" s="36"/>
     </row>
     <row r="57" spans="1:9" ht="15">
       <c r="A57" s="5"/>
@@ -4256,16 +4262,16 @@
       <c r="C57" s="5"/>
       <c r="D57" s="5"/>
       <c r="E57" s="5"/>
-      <c r="F57" s="28" t="s">
-        <v>16</v>
-      </c>
-      <c r="G57" s="28" t="s">
-        <v>16</v>
-      </c>
-      <c r="H57" s="28" t="s">
-        <v>16</v>
-      </c>
-      <c r="I57" s="28" t="s">
+      <c r="F57" s="25" t="s">
+        <v>16</v>
+      </c>
+      <c r="G57" s="25" t="s">
+        <v>16</v>
+      </c>
+      <c r="H57" s="25" t="s">
+        <v>16</v>
+      </c>
+      <c r="I57" s="25" t="s">
         <v>16</v>
       </c>
     </row>
@@ -4275,7 +4281,7 @@
       <c r="C58" s="5"/>
       <c r="D58" s="5"/>
       <c r="E58" s="5"/>
-      <c r="F58" s="29" t="s">
+      <c r="F58" s="26" t="s">
         <v>16</v>
       </c>
       <c r="G58" s="5"/>

</xml_diff>